<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-02 Le carton du marché
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-02.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-02.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Nino, papa</t>
+          <t>Sarah, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut faire entrer le ballon jaune dans le carton du marché. Nino est plus grand, le ballon part sous le banc. Ils rapprochent le carton et jouent ensemble.</t>
+          <t>Une aile sèche tape le banc. Sur l'aile, un éclat de samare brille. Sarah veut le ballon jaune dans le carton, maintenant. Nino est plus grand : il pousse trop haut, le ballon part sous le banc. Sarah refuse de foncer. Ils rapprochent le carton, visent ensemble. Merci vécu. Un éclat de samare reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les samares du tilleul tournent. Elles tombent sur un carton. Le carton sent encore l'orange. Papa le pose près du banc. Un filet dort contre le pied. Dedans, un ballon jaune attend. Tu as vu les samares, Sarah ? Oui, papa. Elles tournent comme des hélices. Oui. Je veux viser le carton. Le ballon dans la boîte ? Oui. En ce moment, Sarah ouvre le filet. Le ballon est un peu froid. Il sent le caoutchouc. Nino arrive près du banc. Nino est plus grand. Sarah est plus petite. Ils ont des tailles différentes. Tu veux le carton avec moi ? Oui. Vous jouez ensemble. On peut jouer ensemble. Sarah pousse le ballon, tout près. Le carton fait un bruit mou. Il est dedans ! Oui. Nino pousse plus fort. Le ballon passe au-dessus. Il roule sous le banc. Il est parti ! On le reprend, tout doux. Sarah se baisse. Son bras passe sous le bois. Nino tient le banc, tout calme. Je le touche ! Doucement. Le ballon revient, un peu poussiéreux. Une samare est collée dessus. Le carton est un peu loin, là. On le rapproche ? Oui.</t>
+          <t>Une aile sèche tape le bois du banc. Elle tourne une fois, puis s'arrête. Elle a tourné, papa. Tu l'as vue, Sarah ? C'est une samare, pâle et légère. Le tilleul ombre le square. Ça sent l'orange, près du carton. C'est le carton du marché. Papa pose le carton près du banc. Le carton est vide, un peu froissé. Il sent l'orange. Les oranges étaient dedans. Un filet dort contre le pied du banc. Dedans, un ballon jaune attend. Il est jaune ! Tu le vois, dans le filet ? Sur l'aile, un éclat de samare brille. Il brille, papa. Tu le vois, sur l'aile ? Sarah touche l'éclat de samare. L'aile est sèche, un peu froide. Elle est froide. Je veux viser le carton, maintenant ! Tu restes près de nous ? Oui, maman. Tu tiens ma manche, Sarah ? Oui, papa. Nino arrive près du banc. Nino est plus grand, près du carton. Sarah est plus petite, contre le bois. Tu viens viser avec moi ? Nino regarde le carton, sans parler. Oui. En ce moment, Sarah ouvre le filet. Le ballon est un peu froid. Il sent le caoutchouc. Il est froid. Je le mets dedans ! Sarah pousse le ballon, tout près. Le carton fait un bruit mou. Il est dedans ! Oui. Nino pousse plus fort, d'en haut. Le ballon passe au-dessus du carton. Il roule sous le banc. Il est parti ! Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Je le prends ! Sarah se baisse trop vite. Son bras cherche, sans voir. Nino tend le bras, trop long. Le ballon recule sous le bois. Je n'arrive pas. Tu le vois, sous le banc ? Papa s'accroupit à la même hauteur. Tes mains sont froides, Sarah ? Un peu, maman. L'herbe est fraîche sous les genoux. Il est loin. On avance.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les samares du tilleul tournent. Elles tombent sur un carton. Le carton sent encore l'orange. Papa le pose près du banc. Un filet dort contre le pied. Dedans, un ballon jaune attend. Tu as vu les samares, Sarah ? Oui, papa. Elles tournent comme des hélices. Oui. Je veux viser le carton. Le ballon dans la boîte ? Oui. En ce moment, Sarah ouvre le filet. Le ballon est un peu froid. Il sent le caoutchouc. Nino arrive près du banc. Nino est plus grand. Sarah est plus petite. Ils ont des tailles différentes. Tu veux le carton avec moi ? Oui. Vous jouez ensemble. On peut jouer ensemble. Sarah pousse le ballon, tout près. Le carton fait un bruit mou. Il est dedans ! Oui. Nino pousse plus fort. Le ballon passe au-dessus. Il roule sous le banc. Il est parti ! On le reprend, tout doux. Sarah se baisse. Son bras passe sous le bois. Nino tient le banc, tout calme. Je le touche ! Doucement. Le ballon revient, un peu poussiéreux. Une samare est collée dessus. Le carton est un peu loin, là. On le rapproche ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une aile sèche tape le bois du banc. Elle tourne une fois, puis s'arrête. Elle a tourné, papa. Tu l'as vue, Sarah ? C'est une samare, pâle et légère. Le tilleul ombre le square. Ça sent l'orange, près du carton. C'est le carton du marché. Papa pose le carton près du banc. Le carton est vide, un peu froissé. Il sent l'orange. Les oranges étaient dedans. Un filet dort contre le pied du banc. Dedans, un ballon jaune attend. Il est jaune ! Tu le vois, dans le filet ? Sur l'aile, un &lt;emphasis level="moderate"&gt;éclat de samare&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur l'aile ? Sarah touche l'éclat de samare. L'aile est sèche, un peu froide. Elle est froide. Je veux viser le carton, maintenant ! Tu restes près de nous ? Oui, maman. Tu tiens ma manche, Sarah ? Oui, papa. Nino arrive près du banc. Nino est plus grand, près du carton. Sarah est plus petite, contre le bois. Tu viens viser avec moi ? Nino regarde le carton, sans parler. Oui. En ce moment, Sarah ouvre le filet. Le ballon est un peu froid. Il sent le caoutchouc. Il est froid. Je le mets dedans ! Sarah pousse le ballon, tout près. Le carton fait un bruit mou. Il est dedans ! Oui. Nino pousse plus fort, d'en haut. Le ballon passe au-dessus du carton. Il roule sous le banc. Il est parti ! Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Je le prends ! Sarah se baisse trop vite. Son bras cherche, sans voir. Nino tend le bras, trop long. Le ballon recule sous le bois. Je n'arrive pas. Tu le vois, sous le banc ? Papa s'accroupit à la même hauteur. Tes mains sont froides, Sarah ? Un peu, maman. L'herbe est fraîche sous les genoux. Il est loin. On avance.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Papa emmène Sami au parc. L'herbe sent la rosée. Un ballon jaune est dans le sac. Lina arrive avec sa maman, puis elle rejoint Sami. Lina est plus grande. Sami est plus petit. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Sami veut jouer au ballon. Il prend le ballon jaune. Papa s'accroupit. Papa dit : les tailles différentes n'empêchent pas le jeu. On invite. On joue ensemble. Sami va vers Lina. Il dit : tu veux le ballon avec moi. Lina dit : oui. Papa montre l'espace de l'herbe, près du banc. Sami tient le ballon contre son ventre. Il le passe tout près. Lina le reçoit. Elle le renvoie plus bas, pour que Sami l'attrape. Le ballon tape les mains de Sami. Il rit. Ils font un cercle. Papa est le troisième. Le ballon va, revient. Parfois Lina saute. Parfois Sami roule le ballon au sol. Les deux façons marchent. Un autre enfant plus grand passe. Il demande le ballon. Sami invite. Ils jouent ensemble à quatre, un moment. Puis le quatrième part. Sami a chaud. Il s'assoit. Lina s'assoit aussi. Papa dit : au bac à sable, vous aviez déjà joué ensemble. Ici, avec le ballon, c'est la même leçon. Petit ou grand, on invite. On joue ensemble. Sami reprend le ballon. Il le pose entre eux. Ils font un but avec deux sacs. Lina garde le but un peu plus loin. Sami tire tout près. Le ballon entre. Ils tapent dans leurs mains. Les tailles différentes sont encore là. Le jeu aussi. [pause]</t>
+          <t>Une aile sèche tape le bois du banc. Elle tourne une fois, puis s'arrête. Elle a tourné, papa. Tu l'as vue, Sarah ? C'est une samare, pâle et légère. Le tilleul ombre le square. Ça sent l'orange, près du carton. C'est le carton du marché. Papa pose le carton près du banc. Le carton est vide, un peu froissé. Il sent l'orange. Les oranges étaient dedans. Un filet dort contre le pied du banc. Dedans, un ballon jaune attend. Il est jaune ! Tu le vois, dans le filet ? Sur l'aile, un &lt;emphasis&gt;éclat de samare&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur l'aile ? Sarah touche l'éclat de samare. L'aile est sèche, un peu froide. Elle est froide. Je veux viser le carton, maintenant ! Tu restes près de nous ? Oui, maman. Tu tiens ma manche, Sarah ? Oui, papa. Nino arrive près du banc. Nino est plus grand, près du carton. Sarah est plus petite, contre le bois. Tu viens viser avec moi ? Nino regarde le carton, sans parler. Oui. En ce moment, Sarah ouvre le filet. Le ballon est un peu froid. Il sent le caoutchouc. Il est froid. Je le mets dedans ! Sarah pousse le ballon, tout près. Le carton fait un bruit mou. Il est dedans ! Oui. Nino pousse plus fort, d'en haut. Le ballon passe au-dessus du carton. Il roule sous le banc. Il est parti ! Oh. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Je le prends ! Sarah se baisse trop vite. Son bras cherche, sans voir. Nino tend le bras, trop long. Le ballon recule sous le bois. Je n'arrive pas. Tu le vois, sous le banc ? Papa s'accroupit à la même hauteur. Tes mains sont froides, Sarah ? Un peu, maman. L'herbe est fraîche sous les genoux. Il est loin. On avance. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de samare</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,52 +1326,77 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_ballon_dans_le_carton_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les samares du tilleul tournent.
-narrateur|Elles tombent sur un carton.
-narrateur|Le carton sent encore l'orange.
-narrateur|Papa le pose près du banc.
-narrateur|Un filet dort contre le pied.
+          <t>narrateur|Une aile sèche tape le bois du banc.
+narrateur|Elle tourne une fois, puis s'arrête.
+enfant-f|Elle a tourné, papa.
+papa|Tu l'as vue, Sarah ?
+narrateur|C'est une samare, pâle et légère.
+narrateur|Le tilleul ombre le square.
+narrateur|Ça sent l'orange, près du carton.
+maman|C'est le carton du marché.
+narrateur|Papa pose le carton près du banc.
+narrateur|Le carton est vide, un peu froissé.
+enfant-f|Il sent l'orange.
+maman|Les oranges étaient dedans.
+narrateur|Un filet dort contre le pied du banc.
 narrateur|Dedans, un ballon jaune attend.
-papa|Tu as vu les samares, Sarah ?
+enfant-f|Il est jaune !
+papa|Tu le vois, dans le filet ?
+narrateur|Sur l'aile, un éclat de samare brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, sur l'aile ?
+narrateur|Sarah touche l'éclat de samare.
+narrateur|L'aile est sèche, un peu froide.
+enfant-f|Elle est froide.
+enfant-f|Je veux viser le carton, maintenant !
+maman|Tu restes près de nous ?
+enfant-f|Oui, maman.
+papa|Tu tiens ma manche, Sarah ?
 enfant-f|Oui, papa.
-enfant-f|Elles tournent comme des hélices.
-papa|Oui.
-enfant-f|Je veux viser le carton.
-papa|Le ballon dans la boîte ?
-enfant-f|Oui.
+narrateur|Nino arrive près du banc.
+narrateur|Nino est plus grand, près du carton.
+narrateur|Sarah est plus petite, contre le bois.
+enfant-f|Tu viens viser avec moi ?
+narrateur|Nino regarde le carton, sans parler.
+enfant-m|Oui.
 narrateur|En ce moment, Sarah ouvre le filet.
 narrateur|Le ballon est un peu froid.
 narrateur|Il sent le caoutchouc.
-narrateur|Nino arrive près du banc.
-narrateur|Nino est plus grand.
-narrateur|Sarah est plus petite.
-narrateur|Ils ont des tailles différentes.
-enfant-f|Tu veux le carton avec moi ?
-copain|Oui.
-papa|Vous jouez ensemble.
-papa|On peut jouer ensemble.
+enfant-f|Il est froid.
+enfant-f|Je le mets dedans !
 narrateur|Sarah pousse le ballon, tout près.
 narrateur|Le carton fait un bruit mou.
 enfant-f|Il est dedans !
 papa|Oui.
-narrateur|Nino pousse plus fort.
-narrateur|Le ballon passe au-dessus.
+narrateur|Nino pousse plus fort, d'en haut.
+narrateur|Le ballon passe au-dessus du carton.
 narrateur|Il roule sous le banc.
 enfant-f|Il est parti !
-papa|On le reprend, tout doux.
-narrateur|Sarah se baisse.
-narrateur|Son bras passe sous le bois.
-narrateur|Nino tient le banc, tout calme.
-enfant-f|Je le touche !
-copain|Doucement.
-narrateur|Le ballon revient, un peu poussiéreux.
-narrateur|Une samare est collée dessus.
-papa|Le carton est un peu loin, là.
-enfant-f|On le rapproche ?
-papa|Oui.</t>
+enfant-m|Oh.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Les épaules de Sarah tombent un peu.
+narrateur|Ça serre, dans son ventre.
+enfant-f|Je le prends !
+narrateur|Sarah se baisse trop vite.
+narrateur|Son bras cherche, sans voir.
+narrateur|Nino tend le bras, trop long.
+narrateur|Le ballon recule sous le bois.
+enfant-f|Je n'arrive pas.
+papa|Tu le vois, sous le banc ?
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont froides, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|L'herbe est fraîche sous les genoux.
+enfant-m|Il est loin.
+papa|On avance.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1408,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah est plus petite. Nino est plus grand. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah est &lt;emphasis level="moderate"&gt;plus petite&lt;/emphasis&gt;. Nino est plus grand. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Sami est plus petit. Lina est plus grande. Que font-ils ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah est &lt;emphasis&gt;plus petite&lt;/emphasis&gt;. Nino est plus grand. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1476,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1484,10 +1509,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1502,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>plus petite</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1538,23 +1567,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=ils_jouent_ensemble_malgre_la_taille; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1588,17 +1617,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah tire le carton, tout près. Nino pousse l'autre bord. Le carton glisse sur l'herbe. Ça sent l'orange encore. Il est tout près, maintenant. Oui. Les deux peuvent viser. Sarah pousse le ballon. Nino le pousse plus bas. Les deux façons marchent. Le ballon entre, deux fois. Encore ! Encore. Vous avez des tailles différentes. Et vous jouez ensemble. C'était bien, le but ? Oui, papa. Un pigeon marche près du filet. Sarah souffle un peu. Nino pose le ballon entre eux. Le carton a un coin froissé. Il a travaillé, le carton. Oui. L'orange aussi, ce matin.</t>
+          <t>Sarah veut le ballon, toute seule. Je le prends, maintenant ! Elle avance trop vite sous le banc. Le ballon glisse plus loin. Oh. Nino veut pousser d'en haut. Je vise fort. Sa main passe au-dessus. Le carton tremble, vide. Il n'entre pas. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme les mains. Elle écoute le square, un instant. Tu veux venir près du carton ? Papa reste à la même hauteur. Sarah pose un pied dans l'herbe. L'herbe est fraîche, un peu mouillée. On le rapproche ? Nino attend, puis prend l'autre bord. Oui. Sarah tire le carton, tout près. Nino pousse l'autre bord. Le carton glisse sur l'herbe. Il sent l'orange. Il est près de vous. Sarah se baisse sous le bois. Son bras court passe sous le banc. Nino tient le banc, plus haut. Je le touche ! Doucement. Le ballon revient, un peu poussiéreux. Une samare est collée dessus. Tu tiens le bord ? Oui. Sarah pousse le ballon, plus bas. Nino le guide, sans le lancer. Le ballon entre, avec un bruit mou. Il est dedans ! Oui. Merci, Sarah. Papa a vu les deux, près du carton. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino, tu tiens le bord ? Oui, papa. Un pigeon marche près du filet. Sarah souffle un peu.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah tire le carton, tout près. Nino pousse l'autre bord. Le carton glisse sur l'herbe. Ça sent l'orange encore. Il est tout près, maintenant. Oui. Les deux peuvent viser. Sarah pousse le ballon. Nino le pousse plus bas. Les deux façons marchent. Le ballon entre, deux fois. Encore ! Encore. Vous avez des tailles différentes. Et vous jouez ensemble. C'était bien, le but ? Oui, papa. Un pigeon marche près du filet. Sarah souffle un peu. Nino pose le ballon entre eux. Le carton a un coin froissé. Il a travaillé, le carton. Oui. L'orange aussi, ce matin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut le ballon, toute seule. Je le prends, maintenant ! Elle avance trop vite sous le banc. Le ballon glisse plus loin. Oh. Nino veut pousser d'en haut. Je vise fort. Sa main passe au-dessus. Le &lt;emphasis level="moderate"&gt;carton&lt;/emphasis&gt; tremble, vide. Il n'entre pas. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme les mains. Elle écoute le square, un instant. Tu veux venir près du carton ? Papa reste à la même hauteur. Sarah pose un pied dans l'herbe. L'herbe est fraîche, un peu mouillée. On le rapproche ? Nino attend, puis prend l'autre bord. Oui. Sarah tire le carton, tout près. Nino pousse l'autre bord. Le carton glisse sur l'herbe. Il sent l'orange. Il est près de vous. Sarah se baisse sous le bois. Son bras court passe sous le banc. Nino tient le banc, plus haut. Je le touche ! Doucement. Le ballon revient, un peu poussiéreux. Une samare est collée dessus. Tu tiens le bord ? Oui. Sarah pousse le ballon, plus bas. Nino le guide, sans le lancer. Le ballon entre, avec un bruit mou. Il est dedans ! Oui. Merci, Sarah. Papa a vu les deux, près du carton. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino, tu tiens le bord ? Oui, papa. Un pigeon marche près du filet. Sarah souffle un peu.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sami a invité. Lina a passé le ballon tout près. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils ont joué ensemble. [pause]</t>
+          <t>Sarah veut le ballon, toute seule. Je le prends, maintenant ! Elle avance trop vite sous le banc. Le ballon glisse plus loin. Oh. Nino veut pousser d'en haut. Je vise fort. Sa main passe au-dessus. Le &lt;emphasis&gt;carton&lt;/emphasis&gt; tremble, vide. Il n'entre pas. Le sourire ne revient pas. Sarah refuse de foncer. Elle referme les mains. Elle écoute le square, un instant. Tu veux venir près du carton ? Papa reste à la même hauteur. Sarah pose un pied dans l'herbe. L'herbe est fraîche, un peu mouillée. On le rapproche ? Nino attend, puis prend l'autre bord. Oui. Sarah tire le carton, tout près. Nino pousse l'autre bord. Le carton glisse sur l'herbe. Il sent l'orange. Il est près de vous. Sarah se baisse sous le bois. Son bras court passe sous le banc. Nino tient le banc, plus haut. Je le touche ! Doucement. Le ballon revient, un peu poussiéreux. Une samare est collée dessus. Tu tiens le bord ? Oui. Sarah pousse le ballon, plus bas. Nino le guide, sans le lancer. Le ballon entre, avec un bruit mou. Il est dedans ! Oui. Merci, Sarah. Papa a vu les deux, près du carton. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Nino, tu tiens le bord ? Oui, papa. Un pigeon marche près du filet. Sarah souffle un peu. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1645,7 +1674,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1653,10 +1682,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1679,7 +1708,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>carton</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1693,16 +1722,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1711,10 +1740,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1727,35 +1756,66 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=le_tir_haut_echoue_le_carton_rapproche_ouvre; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah tire le carton, tout près.
+          <t>narrateur|Sarah veut le ballon, toute seule.
+enfant-f|Je le prends, maintenant !
+narrateur|Elle avance trop vite sous le banc.
+narrateur|Le ballon glisse plus loin.
+enfant-f|Oh.
+narrateur|Nino veut pousser d'en haut.
+enfant-m|Je vise fort.
+narrateur|Sa main passe au-dessus.
+narrateur|Le carton tremble, vide.
+enfant-m|Il n'entre pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme les mains.
+narrateur|Elle écoute le square, un instant.
+papa|Tu veux venir près du carton ?
+narrateur|Papa reste à la même hauteur.
+narrateur|Sarah pose un pied dans l'herbe.
+narrateur|L'herbe est fraîche, un peu mouillée.
+enfant-f|On le rapproche ?
+narrateur|Nino attend, puis prend l'autre bord.
+enfant-m|Oui.
+narrateur|Sarah tire le carton, tout près.
 narrateur|Nino pousse l'autre bord.
 narrateur|Le carton glisse sur l'herbe.
-narrateur|Ça sent l'orange encore.
-enfant-f|Il est tout près, maintenant.
-papa|Oui.
-papa|Les deux peuvent viser.
-narrateur|Sarah pousse le ballon.
-narrateur|Nino le pousse plus bas.
-narrateur|Les deux façons marchent.
-narrateur|Le ballon entre, deux fois.
-copain|Encore !
-enfant-f|Encore.
-papa|Vous avez des tailles différentes.
-papa|Et vous jouez ensemble.
-papa|C'était bien, le but ?
-enfant-f|Oui, papa.
+enfant-f|Il sent l'orange.
+maman|Il est près de vous.
+narrateur|Sarah se baisse sous le bois.
+narrateur|Son bras court passe sous le banc.
+narrateur|Nino tient le banc, plus haut.
+enfant-f|Je le touche !
+enfant-m|Doucement.
+narrateur|Le ballon revient, un peu poussiéreux.
+narrateur|Une samare est collée dessus.
+enfant-f|Tu tiens le bord ?
+enfant-m|Oui.
+narrateur|Sarah pousse le ballon, plus bas.
+narrateur|Nino le guide, sans le lancer.
+narrateur|Le ballon entre, avec un bruit mou.
+enfant-f|Il est dedans !
+enfant-m|Oui.
+papa|Merci, Sarah.
+narrateur|Papa a vu les deux, près du carton.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+papa|Nino, tu tiens le bord ?
+enfant-m|Oui, papa.
 narrateur|Un pigeon marche près du filet.
-narrateur|Sarah souffle un peu.
-narrateur|Nino pose le ballon entre eux.
-narrateur|Le carton a un coin froissé.
-enfant-f|Il a travaillé, le carton.
-papa|Oui.
-papa|L'orange aussi, ce matin.</t>
+narrateur|Sarah souffle un peu.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>carton,herbe</t>
         </is>
       </c>
     </row>
@@ -1782,17 +1842,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range le ballon jaune ? Oui. Papa glisse le ballon dans le filet. Sarah plie le carton, tout doux. Nino ramasse une samare. À demain. À demain. Tu as fini de plier le carton ? Oui, papa. Le tilleul fait encore tourner une hélice. Le banc redevient calme. L'herbe a une trace de carton.</t>
+          <t>Sarah veut un autre but, d'un coup. Je recommence ! Elle tire le ballon trop vite. Nino pousse trop haut, d'élan. Le carton penche sur l'herbe. Oh. Il tombe ! Le ballon sort, puis roule. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Nino attend, sans parler. Personne ne dit la suite. Sarah observe le carton, écoute le square. Sur l'aile, un éclat de samare luit. Là, sur l'aile. Sarah tient le ballon des deux mains. Tu tiens le bord, Nino ? Oui. Nino pose les mains sur le carton. Sarah pousse plus bas, près de l'herbe. Le ballon entre, sans sauter. Il reste dedans. Tu le vois, Sarah ? Oui, papa. On avance ? Oui, maman. Le tilleul laisse une ombre ronde. L'air froid revient sur les joues. J'ai les joues froides. On marche. Sarah passe le long du banc. Le bois craque, un peu. Le carton a un coin froissé. Il a une trace. Il a travaillé, le carton. On laisse le filet ? On le prend.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range le ballon jaune ? Oui. Papa glisse le ballon dans le filet. Sarah plie le carton, tout doux. Nino ramasse une samare. À demain. À demain. Tu as fini de plier le carton ? Oui, papa. Le tilleul fait encore tourner une hélice. Le banc redevient calme. L'herbe a une trace de carton.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah veut un autre but, d'un coup. Je recommence ! Elle tire le ballon trop vite. Nino pousse trop haut, d'élan. Le carton penche sur l'herbe. Oh. Il tombe ! Le ballon sort, puis roule. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Nino attend, sans parler. Personne ne dit la suite. Sarah observe le carton, écoute le square. Sur l'aile, un &lt;emphasis level="moderate"&gt;éclat de samare&lt;/emphasis&gt; luit. Là, sur l'aile. Sarah tient le ballon des deux mains. Tu tiens le bord, Nino ? Oui. Nino pose les mains sur le carton. Sarah pousse plus bas, près de l'herbe. Le ballon entre, sans sauter. Il reste dedans. Tu le vois, Sarah ? Oui, papa. On avance ? Oui, maman. Le tilleul laisse une ombre ronde. L'air froid revient sur les joues. J'ai les joues froides. On marche. Sarah passe le long du banc. Le bois craque, un peu. Le carton a un coin froissé. Il a une trace. Il a travaillé, le carton. On laisse le filet ? On le prend.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range le ballon jaune dans le sac. Sami et Lina se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. Le parc redevient calme. [pause]</t>
+          <t>Sarah veut un autre but, d'un coup. Je recommence ! Elle tire le ballon trop vite. Nino pousse trop haut, d'élan. Le carton penche sur l'herbe. Oh. Il tombe ! Le ballon sort, puis roule. Sarah avance les mains. Puis elle s'arrête net. Attends, je regarde. Nino attend, sans parler. Personne ne dit la suite. Sarah observe le carton, écoute le square. Sur l'aile, un &lt;emphasis&gt;éclat de samare&lt;/emphasis&gt; luit. Là, sur l'aile. Sarah tient le ballon des deux mains. Tu tiens le bord, Nino ? Oui. Nino pose les mains sur le carton. Sarah pousse plus bas, près de l'herbe. Le ballon entre, sans sauter. Il reste dedans. Tu le vois, Sarah ? Oui, papa. On avance ? Oui, maman. Le tilleul laisse une ombre ronde. L'air froid revient sur les joues. J'ai les joues froides. On marche. Sarah passe le long du banc. Le bois craque, un peu. Le carton a un coin froissé. Il a une trace. Il a travaillé, le carton. On laisse le filet ? On le prend. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1839,7 +1899,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1847,10 +1907,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1873,30 +1933,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de samare</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,10 +1965,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1919,21 +1979,51 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|On range le ballon jaune ?
-enfant-f|Oui.
-narrateur|Papa glisse le ballon dans le filet.
-narrateur|Sarah plie le carton, tout doux.
-narrateur|Nino ramasse une samare.
-copain|À demain.
-enfant-f|À demain.
-papa|Tu as fini de plier le carton ?
+          <t>narrateur|Sarah veut un autre but, d'un coup.
+enfant-f|Je recommence !
+narrateur|Elle tire le ballon trop vite.
+narrateur|Nino pousse trop haut, d'élan.
+narrateur|Le carton penche sur l'herbe.
+enfant-f|Oh.
+enfant-m|Il tombe !
+narrateur|Le ballon sort, puis roule.
+narrateur|Sarah avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Nino attend, sans parler.
+narrateur|Personne ne dit la suite.
+narrateur|Sarah observe le carton, écoute le square.
+narrateur|Sur l'aile, un éclat de samare luit.
+enfant-f|Là, sur l'aile.
+narrateur|Sarah tient le ballon des deux mains.
+enfant-f|Tu tiens le bord, Nino ?
+enfant-m|Oui.
+narrateur|Nino pose les mains sur le carton.
+narrateur|Sarah pousse plus bas, près de l'herbe.
+narrateur|Le ballon entre, sans sauter.
+enfant-f|Il reste dedans.
+papa|Tu le vois, Sarah ?
 enfant-f|Oui, papa.
-narrateur|Le tilleul fait encore tourner une hélice.
-narrateur|Le banc redevient calme.
-narrateur|L'herbe a une trace de carton.</t>
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Le tilleul laisse une ombre ronde.
+narrateur|L'air froid revient sur les joues.
+enfant-f|J'ai les joues froides.
+papa|On marche.
+narrateur|Sarah passe le long du banc.
+narrateur|Le bois craque, un peu.
+narrateur|Le carton a un coin froissé.
+enfant-f|Il a une trace.
+maman|Il a travaillé, le carton.
+enfant-m|On laisse le filet ?
+papa|On le prend.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1965,17 +2055,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le ballon est entré. On a joué ensemble. Bravo, Sarah. Le filet est sur l'épaule de papa.</t>
+          <t>L'aile brillait, papa. Tu la vois, comme sur le carton ? Oui, dans l'herbe. Sarah pose le ballon contre le filet. On le glisse dans le filet ? Oui, maman. Le carton sentait l'orange. Il est derrière nous. Une samare n'est plus sur le bois. Sarah respire, plus large. On rentre ? Oui. À demain. À demain. Les joues de Sarah se réchauffent. Le filet est sur l'épaule de papa. Un éclat de samare reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le ballon est entré. On a joué ensemble. Bravo, Sarah. Le filet est sur l'épaule de papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;L'aile brillait, papa. Tu la vois, comme sur le carton ? Oui, dans l'herbe. Sarah pose le ballon contre le filet. On le glisse dans le filet ? Oui, maman. Le carton sentait l'orange. Il est derrière nous. Une samare n'est plus sur le bois. Sarah respire, plus large. On rentre ? Oui. À demain. À demain. Les joues de Sarah se réchauffent. Le filet est sur l'épaule de papa. Un &lt;emphasis level="moderate"&gt;éclat de samare&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'aile brillait, papa. Tu la vois, comme sur le carton ? Oui, dans l'herbe. Sarah pose le ballon contre le filet. On le glisse dans le filet ? Oui, maman. Le carton sentait l'orange. Il est derrière nous. Une samare n'est plus sur le bois. Sarah respire, plus large. On rentre ? Oui. À demain. À demain. Les joues de Sarah se réchauffent. Le filet est sur l'épaule de papa. Un &lt;emphasis&gt;éclat de samare&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2022,15 +2112,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2042,12 +2132,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2056,17 +2146,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de samare</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2075,11 +2169,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2088,27 +2182,44 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le ballon est entré.
-enfant-f|On a joué ensemble.
-papa|Bravo, Sarah.
-narrateur|Le filet est sur l'épaule de papa.</t>
+          <t>enfant-f|L'aile brillait, papa.
+papa|Tu la vois, comme sur le carton ?
+enfant-f|Oui, dans l'herbe.
+narrateur|Sarah pose le ballon contre le filet.
+maman|On le glisse dans le filet ?
+enfant-f|Oui, maman.
+enfant-f|Le carton sentait l'orange.
+maman|Il est derrière nous.
+narrateur|Une samare n'est plus sur le bois.
+narrateur|Sarah respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+enfant-m|À demain.
+enfant-f|À demain.
+narrateur|Les joues de Sarah se réchauffent.
+narrateur|Le filet est sur l'épaule de papa.
+narrateur|Un éclat de samare reste pâle.</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2207,6 +2318,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>